<commit_message>
Actualizacao dos dados financeiros
</commit_message>
<xml_diff>
--- a/EMPREENDEDORAS_PAM_VERDE_C3_2026.xlsx
+++ b/EMPREENDEDORAS_PAM_VERDE_C3_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://muvamozorg.sharepoint.com/sites/mis.drive/Documentos Partilhados/PROJECTOS/Sistema de Monitoria/Pam_Verde/2026/Baseline_Endline/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="225" documentId="11_0DFBC18E49307CB38E73D6987E34D4946C7A7096" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D722354E-BFC5-4D44-9CC1-B7C001EF276D}"/>
+  <xr:revisionPtr revIDLastSave="227" documentId="11_0DFBC18E49307CB38E73D6987E34D4946C7A7096" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A74B5B17-BBE3-4152-AAAE-83EBE1C8126C}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Empreendedoras_Nampula_C3_2026" sheetId="1" r:id="rId1"/>
@@ -17863,12 +17863,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="20d57abc-823c-4051-a81a-1a0a01a8f39e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -18107,20 +18109,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="20d57abc-823c-4051-a81a-1a0a01a8f39e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5422FBB-6025-4E11-8C1C-C4A520C0A5F3}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6C6D4B0-20F6-407F-B938-614BBBC09F61}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="54c5ab46-7543-4aba-b0fa-79d6a199bef5"/>
+    <ds:schemaRef ds:uri="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -18145,12 +18148,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6C6D4B0-20F6-407F-B938-614BBBC09F61}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5422FBB-6025-4E11-8C1C-C4A520C0A5F3}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="54c5ab46-7543-4aba-b0fa-79d6a199bef5"/>
-    <ds:schemaRef ds:uri="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Calculos actualizados do grafico servicos e botoes png
</commit_message>
<xml_diff>
--- a/EMPREENDEDORAS_PAM_VERDE_C3_2026.xlsx
+++ b/EMPREENDEDORAS_PAM_VERDE_C3_2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://muvamozorg.sharepoint.com/sites/mis.drive/Documentos Partilhados/PROJECTOS/Sistema de Monitoria/Pam_Verde/2026/Baseline_Endline/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="227" documentId="11_0DFBC18E49307CB38E73D6987E34D4946C7A7096" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A74B5B17-BBE3-4152-AAAE-83EBE1C8126C}"/>
+  <xr:revisionPtr revIDLastSave="230" documentId="11_0DFBC18E49307CB38E73D6987E34D4946C7A7096" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DCA3AEC7-E457-45A3-9060-796FE3D0B851}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17863,14 +17863,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="20d57abc-823c-4051-a81a-1a0a01a8f39e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -18109,21 +18107,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="20d57abc-823c-4051-a81a-1a0a01a8f39e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6C6D4B0-20F6-407F-B938-614BBBC09F61}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5422FBB-6025-4E11-8C1C-C4A520C0A5F3}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="54c5ab46-7543-4aba-b0fa-79d6a199bef5"/>
-    <ds:schemaRef ds:uri="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -18148,9 +18145,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5422FBB-6025-4E11-8C1C-C4A520C0A5F3}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6C6D4B0-20F6-407F-B938-614BBBC09F61}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="54c5ab46-7543-4aba-b0fa-79d6a199bef5"/>
+    <ds:schemaRef ds:uri="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>